<commit_message>
Roll Scorecard up to regulation-family categories
Scorecard sheet now shows one row per regulation FAMILY instead of one
per specific citation. Columns are:
    Regulation | What it means | # Unique Citations | # Contracts | Contract IDs

On the current 39-contract demo the sheet drops from 60 rows to 10
rows: FAR, DFARS, DLAD, NMCARS, JAR, HSAR, NFS, CFR, USC, EO. Each
row aggregates every KEPT citation from that family (dropped
boilerplate still applies).

Per-citation detail is preserved on:
  - Contract x Clause  (which specific citation appeared in which contract)
  - Dropped Clauses    (which specific citations the filter removed and why)

clause_extractor.REGULATION_DESCRIPTIONS: one-line description of each
regulation family for the new "What it means" column, covering all
supplements + new citation classes (CFR, USC, EO, DoDI/M/D, PubL).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DjYiNisoHf5A9dZxUQ422r
</commit_message>
<xml_diff>
--- a/supplier_scorecard/output/supplier_scorecard.xlsx
+++ b/supplier_scorecard/output/supplier_scorecard.xlsx
@@ -569,44 +569,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Citation</t>
+          <t>Regulation</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Part</t>
+          <t>What it means</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t># Unique Citations</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>What it means</t>
+          <t># Contracts</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Contract IDs</t>
         </is>
@@ -615,58 +609,44 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>FAR 52.212-4</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>52.212</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>Contract Terms and Conditions—Commercial Products and Commercial Services</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>The standard commercial-item contract terms: payment, inspection, warranty, disputes.</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE7LX26D0059, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>DoD's FAR supplement — cybersecurity (NIST 800-171 / CMMC), sourcing (specialty metals, Buy American), tech-data rights, item marking.</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE7LX26D0059, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FAR 52.212-5</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>52.212</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Contract Terms and Conditions Required to Implement Statutes or Executive Orders—Commercial Products and Commercial Services</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>The list of statutorily required clauses that also apply to commercial contracts (EEO, small-business, labor, etc.).</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="n">
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Federal Acquisition Regulation — baseline procurement rules for every US federal contract.</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="D3" s="8" t="n">
         <v>39</v>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE7LX26D0059, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
         </is>
@@ -675,1708 +655,184 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>FAR 52.243-1</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>52.243</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Changes—Fixed-Price</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Changes clause — the CO may unilaterally change certain contract terms; you get an equitable adjustment.</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE7LX26D0059, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+          <t>DLAD</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Defense Logistics Agency directive — supply-chain-focused clauses (delivery, higher-level QMS, source inspection, item-peculiar packaging) applied to every DLA solicitation.</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FAR 52.249-8</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>52.249</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Default (Fixed-Price Supply and Service)</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Default clause — government may terminate for cause; you may be liable for excess reprocurement costs.</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="n">
-        <v>39</v>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE7LX26D0059, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+          <t>NFS</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>NASA FAR Supplement — mission-critical safety, IT security, export licensing, and patent-rights clauses.</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-DetaClad_Explosion_Clad_Metal_made_up_of</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>FAR 52.204-24</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>52.204</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Representation Regarding Certain Telecommunications and Video Surveillance Services or Equipment</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Represent whether you use covered Chinese telecom (Huawei, ZTE, Hytera, Hikvision, Dahua).</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>38</v>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+          <t>NMCARS</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Navy / Marine Corps FAR supplement — Navy-specific facility access, accident reporting, and technical-instruction clauses.</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FAR 52.204-25</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>52.204</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Prohibition on Contracting for Certain Telecommunications and Video Surveillance Services or Equipment</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Section 889 — you cannot provide the government any covered Chinese telecom equipment/services.</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="n">
-        <v>38</v>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+          <t>HSAR</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>DHS Homeland Security Acquisition Regulation — DHS-specific IT security and contractor-employee access clauses.</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-OEM_Reverse_Osmosis_Unit</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>FAR 52.212-1</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>52.212</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Instructions to Offerors—Commercial Products and Commercial Services</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Standard offer instructions for commercial-item solicitations (how and when to submit your bid).</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>38</v>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+          <t>CFR</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Code of Federal Regulations — direct citations of regulatory schemes (ITAR at 22 CFR 120–130, EAR at 15 CFR 730–774, SBA size at 13 CFR 121, etc.).</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, SPE7L126T679S, SPE7L126T681K, SPE7L326Q1121, SPE7L326T035G, SPE7L326T061D, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5040, SPE7L426T5042, SPE7L726T3634</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FAR 52.225-1</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>52.225</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Buy American—Supplies</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Buy American Act — supply end items must be domestic (or from a qualifying country).</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="n">
-        <v>38</v>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+          <t>JAR</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>DoJ Acquisition Regulation — DoJ-specific employee security screening and OCI/standards-of-conduct clauses.</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-Suppressors_5.56_NATO</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>FAR 52.246-2</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>52.246</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Inspection of Supplies—Fixed-Price</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Inspection of Supplies — you're responsible for QC; government inspects at destination (or origin if specified).</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>38</v>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+          <t>EO</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Executive Orders — presidential directives with cross-cutting supplier obligations (EO 14028 Cybersecurity, EO 14026 Federal Contractor $17.20 Min Wage, EO 13706 Paid Sick Leave, etc.).</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FAR 52.247-34</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>52.247</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>F.o.b. Destination</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>F.o.b. Destination — you own the freight cost and risk of loss until delivery.</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="n">
-        <v>38</v>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>DFARS 252.204-7012</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>252.204</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Safeguarding Covered Defense Information and Cyber Incident Reporting</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Safeguard Covered Defense Information per NIST SP 800-171; report cyber incidents to DoD within 72 hours.</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="n">
-        <v>36</v>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE7LX26D0059, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>DFARS 252.204-7019</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>252.204</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Notice of NIST SP 800-171 DoD Assessment Requirements</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>You must have posted a NIST SP 800-171 self-assessment score in SPRS before award.</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="n">
+          <t>USC</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>United States Code — statutory basis for many FAR/DFARS clauses (Berry Amendment 10 USC 4862, Specialty Metals 10 USC 4863, Buy American 41 USC 8302, etc.).</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>DFARS 252.204-7020</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>252.204</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>NIST SP 800-171 DoD Assessment Requirements</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>You must provide NIST 800-171 assessment info on request; DoD may conduct Medium/High assessments.</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>DFARS 252.204-7021</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>252.204</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Contractor Compliance with the Cybersecurity Maturity Model Certification Level Requirement</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>You must hold the required CMMC certification level before award.</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="n">
-        <v>35</v>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>DFARS 252.211-7003</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>252.211</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Item Unique Identification and Valuation</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Mark deliverables with an Item Unique Identifier (IUID) per MIL-STD-130; register in the DoD IUID registry.</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>DFARS 252.225-7000</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>252.225</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>Buy American—Balance of Payments Program Certificate</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>Certify country of origin for supplies (Buy American / Balance of Payments certificate).</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="n">
-        <v>35</v>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>DFARS 252.225-7001</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>252.225</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Buy American and Balance of Payments Program</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Provide only domestic or qualifying-country end products (DoD Buy American).</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>DFARS 252.225-7002</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>252.225</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>Qualifying Country Sources as Subcontractors</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>Your subcontractors must also source from the US or qualifying countries.</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="n">
-        <v>35</v>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>DFARS 252.225-7012</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>252.225</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Preference for Certain Domestic Commodities</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Certain commodities (food, hand tools, some chemicals) must be domestic — 'Preference for Certain Domestic Commodities.'</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>DFARS 252.227-7013</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>252.227</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Rights in Technical Data—Noncommercial Items</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>Government gets a license to noncommercial technical data you deliver.</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="n">
-        <v>35</v>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>DFARS 252.227-7015</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>252.227</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Technical Data—Commercial Items</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Government gets a license to commercial technical data you deliver.</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>DFARS 252.243-7001</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>252.243</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Pricing of Contract Modifications</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>Contract modifications are priced per Truth in Negotiations Act (cost or pricing data).</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="n">
-        <v>35</v>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>DFARS 252.244-7000</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>252.244</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Subcontracts for Commercial Products or Commercial Services</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Flow the same requirements down to your commercial-item subcontractors.</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>DFARS 252.247-7023</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>252.247</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>Transportation of Supplies by Sea</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>Ocean shipments must move on US-flag vessels to the extent available.</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="n">
-        <v>35</v>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>DLAD 52.211-9006</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>52.211</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Time of Delivery</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>DLA delivery schedule — dictates required leadtime from contract award to shipment.</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>DLAD 52.215-9016</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>52.215</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>Technical and Quality Requirements</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>Higher-level technical and quality requirements may apply (e.g., ISO 9001, AS9100).</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="n">
-        <v>35</v>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>DLAD 52.246-9008</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>52.246</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Inspection and Acceptance at Origin</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>Inspection and acceptance is at origin (source inspection at your facility).</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>DLAD 52.246-9012</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>52.246</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>Higher-Level Contract Quality Requirements</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>Implement a higher-level quality management system (typically ISO 9001 or AS9100).</t>
-        </is>
-      </c>
-      <c r="E29" s="8" t="n">
-        <v>35</v>
-      </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>DLAD 52.246-9080</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>52.246</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>Quality System — DLA-Managed Items</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>DLA-managed items have specific quality-system requirements you must meet.</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>DLAD 52.247-9032</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>52.247</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>Item Peculiar Packaging and Marking</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>Item-peculiar packaging and marking — DLA-specific packing/marking specs.</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="n">
-        <v>35</v>
-      </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>EO 14028</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>14028</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr"/>
-      <c r="D32" s="5" t="inlineStr"/>
-      <c r="E32" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>USC 10.4862</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>10.4862</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr"/>
-      <c r="D33" s="7" t="inlineStr"/>
-      <c r="E33" s="8" t="n">
-        <v>35</v>
-      </c>
-      <c r="F33" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>CFR 15.730-774</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>15.730</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr"/>
-      <c r="D34" s="5" t="inlineStr"/>
-      <c r="E34" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, SPE7L126T679S, SPE7L126T681K, SPE7L326Q1121, SPE7L326T035G, SPE7L326T061D, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5040, SPE7L426T5042, SPE7L726T3634</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>CFR 22.120-130</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>22.120</t>
-        </is>
-      </c>
-      <c r="C35" s="7" t="inlineStr"/>
-      <c r="D35" s="7" t="inlineStr"/>
-      <c r="E35" s="8" t="n">
-        <v>13</v>
-      </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, SPE7L126T679S, SPE7L126T681K, SPE7L326Q1121, SPE7L326T035G, SPE7L326T061D, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5040, SPE7L426T5042, SPE7L726T3634</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>DFARS 252.225-7048</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>252.225</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>Export-Controlled Items</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Comply with ITAR/EAR export-control laws; obtain any required licenses.</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, SPE7L126T679S, SPE7L126T681K, SPE7L326Q1121, SPE7L326T035G, SPE7L326T061D, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5040, SPE7L426T5042, SPE7L726T3634</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>DFARS 252.223-7008</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>252.223</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>Prohibition of Hexavalent Chromium</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>No hexavalent chromium in deliverables unless the CO approves in writing.</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="F37" s="7" t="inlineStr">
-        <is>
-          <t>SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>DFARS 252.225-7008</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>252.225</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>Restriction on Acquisition of Specialty Metals</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>Use only domestically melted or produced specialty metals unless an exception applies.</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>DFARS 252.225-7009</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>252.225</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>Restriction on Acquisition of Certain Articles Containing Specialty Metals</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>Restriction on foreign specialty metals in items with specialty-metal content.</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E926T2719</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>DFARS 252.239-7018</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>252.239</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>Supply Chain Risk</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Assess and mitigate supply-chain risk (SCRM) across your supplier tiers.</t>
-        </is>
-      </c>
-      <c r="E40" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>SPE7L426T4775, SPE7L426T5040, SPE7L426T5042</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>DFARS 252.246-7003</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>252.246</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>Notification of Potential Safety Issues</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>Notify DoD promptly of any safety issue discovered with a delivered item.</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>SPE7L426T4775, SPE7L426T5040, SPE7L426T5042</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>DFARS 252.246-7008</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>252.246</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>Sources of Electronic Parts</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Source electronic parts from OEMs, franchised dealers, or trusted suppliers — no unauthorized brokers.</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>SPE7L426T4775, SPE7L426T5040, SPE7L426T5042</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>NMCARS 5252.204-9400</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>5252.204</t>
-        </is>
-      </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>Contractor Access to Federally-Controlled Facilities</t>
-        </is>
-      </c>
-      <c r="D43" s="7" t="inlineStr">
-        <is>
-          <t>Navy contractor access to federally-controlled facilities.</t>
-        </is>
-      </c>
-      <c r="E43" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>NMCARS 5252.222-9300</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>5252.222</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>Contractor Personnel Access to Work Sites</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Navy contractor personnel access to Navy work sites.</t>
-        </is>
-      </c>
-      <c r="E44" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F44" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>NMCARS 5252.223-9400</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>5252.223</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="inlineStr">
-        <is>
-          <t>Accident Reporting and Investigation</t>
-        </is>
-      </c>
-      <c r="D45" s="7" t="inlineStr">
-        <is>
-          <t>Report accidents/incidents to the Navy per this clause.</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F45" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>NMCARS 5252.242-9115</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>5252.242</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>Technical Instructions</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>Comply with technical instructions issued during performance.</t>
-        </is>
-      </c>
-      <c r="E46" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F46" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>FAR 52.219-14</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>52.219</t>
-        </is>
-      </c>
-      <c r="C47" s="7" t="inlineStr">
-        <is>
-          <t>Limitations on Subcontracting</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>As a set-aside prime, you must perform at least 50% of the cost of manufacture with your own employees (supply contracts).</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-Suppressors_5.56_NATO</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>FAR 52.219-28</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>52.219</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>Post-Award Small Business Program Rerepresentation</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Re-represent your small-business size if you outgrow the standard during performance.</t>
-        </is>
-      </c>
-      <c r="E48" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-Suppressors_5.56_NATO</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>FAR 52.219-6</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>52.219</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="inlineStr">
-        <is>
-          <t>Notice of Total Small Business Set-Aside</t>
-        </is>
-      </c>
-      <c r="D49" s="7" t="inlineStr">
-        <is>
-          <t>This procurement is set aside for small business — only SBs may bid.</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-Suppressors_5.56_NATO</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>FAR 52.219-8</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>52.219</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>Utilization of Small Business Concerns</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>Give small business and socioeconomic categories equitable subcontract opportunity.</t>
-        </is>
-      </c>
-      <c r="E50" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-Suppressors_5.56_NATO</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>HSAR 3052.204-70</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>3052.204</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>Security Requirements for Unclassified Information Technology Resources</t>
-        </is>
-      </c>
-      <c r="D51" s="7" t="inlineStr">
-        <is>
-          <t>DHS IT-resources security requirements.</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-OEM_Reverse_Osmosis_Unit</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>HSAR 3052.204-71</t>
-        </is>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>3052.204</t>
-        </is>
-      </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>Contractor Employee Access</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>DHS contractor-employee access clearance.</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F52" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-OEM_Reverse_Osmosis_Unit</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>HSAR 3052.219-70</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>3052.219</t>
-        </is>
-      </c>
-      <c r="C53" s="7" t="inlineStr">
-        <is>
-          <t>Small Business Subcontracting Plan Reporting</t>
-        </is>
-      </c>
-      <c r="D53" s="7" t="inlineStr">
-        <is>
-          <t>Small-business subcontracting-plan reporting for DHS.</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F53" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-OEM_Reverse_Osmosis_Unit</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>JAR 2852.204-70</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>2852.204</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>Contractor Employee Security Screening</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>DoJ contractor employees must undergo security screening.</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F54" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-Suppressors_5.56_NATO</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>JAR 2852.209-71</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>2852.209</t>
-        </is>
-      </c>
-      <c r="C55" s="7" t="inlineStr">
-        <is>
-          <t>Standards of Conduct</t>
-        </is>
-      </c>
-      <c r="D55" s="7" t="inlineStr">
-        <is>
-          <t>DoJ standards of conduct — apply to your on-site employees.</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-Suppressors_5.56_NATO</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>NFS 1852.204-76</t>
-        </is>
-      </c>
-      <c r="B56" s="4" t="inlineStr">
-        <is>
-          <t>1852.204</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>Security Requirements for Unclassified Information Technology Resources</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>NASA IT-security requirements for unclassified systems.</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F56" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-DetaClad_Explosion_Clad_Metal_made_up_of</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>NFS 1852.223-70</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>1852.223</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="inlineStr">
-        <is>
-          <t>Safety and Health</t>
-        </is>
-      </c>
-      <c r="D57" s="7" t="inlineStr">
-        <is>
-          <t>Maintain a written Safety and Health plan.</t>
-        </is>
-      </c>
-      <c r="E57" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F57" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-DetaClad_Explosion_Clad_Metal_made_up_of</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>NFS 1852.225-70</t>
-        </is>
-      </c>
-      <c r="B58" s="4" t="inlineStr">
-        <is>
-          <t>1852.225</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>Export Licenses</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Handle export licensing for items subject to ITAR/EAR.</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F58" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-DetaClad_Explosion_Clad_Metal_made_up_of</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>NFS 1852.227-11</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>1852.227</t>
-        </is>
-      </c>
-      <c r="C59" s="7" t="inlineStr">
-        <is>
-          <t>Patent Rights — Ownership by the Contractor</t>
-        </is>
-      </c>
-      <c r="D59" s="7" t="inlineStr">
-        <is>
-          <t>Contractor may retain title to inventions (Bayh-Dole implementation).</t>
-        </is>
-      </c>
-      <c r="E59" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F59" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-DetaClad_Explosion_Clad_Metal_made_up_of</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="4" t="inlineStr">
-        <is>
-          <t>NFS 1852.245-70</t>
-        </is>
-      </c>
-      <c r="B60" s="4" t="inlineStr">
-        <is>
-          <t>1852.245</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>Contractor Requests for Government-Owned Equipment</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>Rules for requesting and using NASA-owned equipment.</t>
-        </is>
-      </c>
-      <c r="E60" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F60" s="5" t="inlineStr">
-        <is>
-          <t>MOCK-DetaClad_Explosion_Clad_Metal_made_up_of</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>NFS 1852.246-70</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>1852.246</t>
-        </is>
-      </c>
-      <c r="C61" s="7" t="inlineStr">
-        <is>
-          <t>Mission Critical Space System Personnel Reliability Program</t>
-        </is>
-      </c>
-      <c r="D61" s="7" t="inlineStr">
-        <is>
-          <t>Mission-critical space system personnel reliability program.</t>
-        </is>
-      </c>
-      <c r="E61" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F61" s="7" t="inlineStr">
-        <is>
-          <t>MOCK-DetaClad_Explosion_Clad_Metal_made_up_of</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 'Citation Detail' sheet — per-citation drilldown under Scorecard
Restores the pre-rollup per-citation view as a dedicated sheet
positioned right after the rolled-up Scorecard. Columns:

    Regulation | Citation | Part | Title | What it means | Count | Contract IDs

Rows sorted by (regulation asc, count desc, number asc), so each
regulation family is a contiguous block. The first row of each new
regulation is bolded so the sections read as clear groups.

Only KEPT citations appear — dropped boilerplate still has its own
"Dropped Clauses" sheet.

Workbook sheet order is now:
  Scorecard          (10 rows — one per regulation family)
  Citation Detail    (60 rows — every kept citation, grouped)
  Contract x Clause  (60 × 39 matrix)
  MIL-Specs & Standards
  Raw Contracts
  Dropped Clauses

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DjYiNisoHf5A9dZxUQ422r
</commit_message>
<xml_diff>
--- a/supplier_scorecard/output/supplier_scorecard.xlsx
+++ b/supplier_scorecard/output/supplier_scorecard.xlsx
@@ -9,10 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="!! SIMULATED DATA !!" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorecard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contract x Clause" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MIL-Specs &amp; Standards" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Contracts" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dropped Clauses" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Citation Detail" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contract x Clause" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MIL-Specs &amp; Standards" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Contracts" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dropped Clauses" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +41,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -77,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -99,6 +103,13 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -847,6 +858,2134 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Regulation</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Citation</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>What it means</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Contract IDs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>CFR</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>CFR 15.730-774</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>15.730</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr"/>
+      <c r="E2" s="10" t="inlineStr"/>
+      <c r="F2" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, SPE7L126T679S, SPE7L126T681K, SPE7L326Q1121, SPE7L326T035G, SPE7L326T061D, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5040, SPE7L426T5042, SPE7L726T3634</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CFR</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CFR 22.120-130</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>22.120</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, SPE7L126T679S, SPE7L126T681K, SPE7L326Q1121, SPE7L326T035G, SPE7L326T061D, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5040, SPE7L426T5042, SPE7L726T3634</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>DFARS 252.204-7012</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>252.204</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Safeguarding Covered Defense Information and Cyber Incident Reporting</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Safeguard Covered Defense Information per NIST SP 800-171; report cyber incidents to DoD within 72 hours.</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>36</v>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE7LX26D0059, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DFARS 252.204-7019</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>252.204</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Notice of NIST SP 800-171 DoD Assessment Requirements</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>You must have posted a NIST SP 800-171 self-assessment score in SPRS before award.</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>DFARS 252.204-7020</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>252.204</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>NIST SP 800-171 DoD Assessment Requirements</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>You must provide NIST 800-171 assessment info on request; DoD may conduct Medium/High assessments.</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DFARS 252.204-7021</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>252.204</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Contractor Compliance with the Cybersecurity Maturity Model Certification Level Requirement</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>You must hold the required CMMC certification level before award.</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>DFARS 252.211-7003</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>252.211</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Item Unique Identification and Valuation</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Mark deliverables with an Item Unique Identifier (IUID) per MIL-STD-130; register in the DoD IUID registry.</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DFARS 252.225-7000</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>252.225</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Buy American—Balance of Payments Program Certificate</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Certify country of origin for supplies (Buy American / Balance of Payments certificate).</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>DFARS 252.225-7001</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>252.225</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Buy American and Balance of Payments Program</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Provide only domestic or qualifying-country end products (DoD Buy American).</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DFARS 252.225-7002</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>252.225</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Qualifying Country Sources as Subcontractors</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Your subcontractors must also source from the US or qualifying countries.</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>DFARS 252.225-7012</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>252.225</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Preference for Certain Domestic Commodities</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Certain commodities (food, hand tools, some chemicals) must be domestic — 'Preference for Certain Domestic Commodities.'</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>DFARS 252.227-7013</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>252.227</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Rights in Technical Data—Noncommercial Items</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Government gets a license to noncommercial technical data you deliver.</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>DFARS 252.227-7015</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>252.227</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Technical Data—Commercial Items</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Government gets a license to commercial technical data you deliver.</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>DFARS 252.243-7001</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>252.243</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Pricing of Contract Modifications</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Contract modifications are priced per Truth in Negotiations Act (cost or pricing data).</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>DFARS 252.244-7000</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>252.244</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Subcontracts for Commercial Products or Commercial Services</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Flow the same requirements down to your commercial-item subcontractors.</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>DFARS 252.247-7023</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>252.247</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Transportation of Supplies by Sea</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Ocean shipments must move on US-flag vessels to the extent available.</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>DFARS 252.225-7048</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>252.225</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Export-Controlled Items</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Comply with ITAR/EAR export-control laws; obtain any required licenses.</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, SPE7L126T679S, SPE7L126T681K, SPE7L326Q1121, SPE7L326T035G, SPE7L326T061D, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5040, SPE7L426T5042, SPE7L726T3634</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>DFARS 252.223-7008</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>252.223</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Prohibition of Hexavalent Chromium</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>No hexavalent chromium in deliverables unless the CO approves in writing.</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>DFARS 252.225-7008</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>252.225</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Restriction on Acquisition of Specialty Metals</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Use only domestically melted or produced specialty metals unless an exception applies.</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>DFARS 252.225-7009</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>252.225</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Restriction on Acquisition of Certain Articles Containing Specialty Metals</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Restriction on foreign specialty metals in items with specialty-metal content.</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>DFARS 252.239-7018</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>252.239</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Supply Chain Risk</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Assess and mitigate supply-chain risk (SCRM) across your supplier tiers.</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>SPE7L426T4775, SPE7L426T5040, SPE7L426T5042</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>DFARS 252.246-7003</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>252.246</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Notification of Potential Safety Issues</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Notify DoD promptly of any safety issue discovered with a delivered item.</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>SPE7L426T4775, SPE7L426T5040, SPE7L426T5042</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>DFARS</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>DFARS 252.246-7008</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>252.246</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Sources of Electronic Parts</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Source electronic parts from OEMs, franchised dealers, or trusted suppliers — no unauthorized brokers.</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>SPE7L426T4775, SPE7L426T5040, SPE7L426T5042</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>DLAD</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>DLAD 52.211-9006</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>52.211</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>Time of Delivery</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>DLA delivery schedule — dictates required leadtime from contract award to shipment.</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>DLAD</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>DLAD 52.215-9016</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>52.215</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Technical and Quality Requirements</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Higher-level technical and quality requirements may apply (e.g., ISO 9001, AS9100).</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>DLAD</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>DLAD 52.246-9008</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>52.246</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Inspection and Acceptance at Origin</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Inspection and acceptance is at origin (source inspection at your facility).</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>DLAD</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>DLAD 52.246-9012</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>52.246</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Higher-Level Contract Quality Requirements</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Implement a higher-level quality management system (typically ISO 9001 or AS9100).</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>DLAD</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>DLAD 52.246-9080</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>52.246</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Quality System — DLA-Managed Items</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>DLA-managed items have specific quality-system requirements you must meet.</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>DLAD</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>DLAD 52.247-9032</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>52.247</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Item Peculiar Packaging and Marking</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Item-peculiar packaging and marking — DLA-specific packing/marking specs.</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>EO</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>EO 14028</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>14028</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr"/>
+      <c r="E31" s="10" t="inlineStr"/>
+      <c r="F31" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>FAR 52.212-4</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>52.212</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>Contract Terms and Conditions—Commercial Products and Commercial Services</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>The standard commercial-item contract terms: payment, inspection, warranty, disputes.</t>
+        </is>
+      </c>
+      <c r="F32" s="11" t="n">
+        <v>39</v>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE7LX26D0059, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>FAR 52.212-5</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>52.212</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Contract Terms and Conditions Required to Implement Statutes or Executive Orders—Commercial Products and Commercial Services</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>The list of statutorily required clauses that also apply to commercial contracts (EEO, small-business, labor, etc.).</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="n">
+        <v>39</v>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE7LX26D0059, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>FAR 52.243-1</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>52.243</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Changes—Fixed-Price</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Changes clause — the CO may unilaterally change certain contract terms; you get an equitable adjustment.</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE7LX26D0059, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>FAR 52.249-8</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>52.249</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Default (Fixed-Price Supply and Service)</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Default clause — government may terminate for cause; you may be liable for excess reprocurement costs.</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="n">
+        <v>39</v>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE7LX26D0059, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>FAR 52.204-24</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>52.204</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Representation Regarding Certain Telecommunications and Video Surveillance Services or Equipment</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Represent whether you use covered Chinese telecom (Huawei, ZTE, Hytera, Hikvision, Dahua).</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>FAR 52.204-25</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>52.204</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Prohibition on Contracting for Certain Telecommunications and Video Surveillance Services or Equipment</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Section 889 — you cannot provide the government any covered Chinese telecom equipment/services.</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>FAR 52.212-1</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>52.212</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Instructions to Offerors—Commercial Products and Commercial Services</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Standard offer instructions for commercial-item solicitations (how and when to submit your bid).</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>FAR 52.225-1</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>52.225</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Buy American—Supplies</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Buy American Act — supply end items must be domestic (or from a qualifying country).</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>FAR 52.246-2</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>52.246</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Inspection of Supplies—Fixed-Price</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Inspection of Supplies — you're responsible for QC; government inspects at destination (or origin if specified).</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>FAR 52.247-34</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>52.247</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>F.o.b. Destination</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>F.o.b. Destination — you own the freight cost and risk of loss until delivery.</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-DetaClad_Explosion_Clad_Metal_made_up_of, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-OEM_Reverse_Osmosis_Unit, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Suppressors_5.56_NATO, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>FAR 52.219-14</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>52.219</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Limitations on Subcontracting</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>As a set-aside prime, you must perform at least 50% of the cost of manufacture with your own employees (supply contracts).</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-Suppressors_5.56_NATO</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>FAR 52.219-28</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>52.219</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Post-Award Small Business Program Rerepresentation</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>Re-represent your small-business size if you outgrow the standard during performance.</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-Suppressors_5.56_NATO</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>FAR 52.219-6</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>52.219</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Notice of Total Small Business Set-Aside</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>This procurement is set aside for small business — only SBs may bid.</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-Suppressors_5.56_NATO</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>FAR</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>FAR 52.219-8</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>52.219</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Utilization of Small Business Concerns</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Give small business and socioeconomic categories equitable subcontract opportunity.</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-Suppressors_5.56_NATO</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>HSAR</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>HSAR 3052.204-70</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>3052.204</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>Security Requirements for Unclassified Information Technology Resources</t>
+        </is>
+      </c>
+      <c r="E46" s="10" t="inlineStr">
+        <is>
+          <t>DHS IT-resources security requirements.</t>
+        </is>
+      </c>
+      <c r="F46" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="10" t="inlineStr">
+        <is>
+          <t>MOCK-OEM_Reverse_Osmosis_Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>HSAR</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>HSAR 3052.204-71</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>3052.204</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Contractor Employee Access</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>DHS contractor-employee access clearance.</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-OEM_Reverse_Osmosis_Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>HSAR</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>HSAR 3052.219-70</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>3052.219</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Small Business Subcontracting Plan Reporting</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Small-business subcontracting-plan reporting for DHS.</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-OEM_Reverse_Osmosis_Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>JAR</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>JAR 2852.204-70</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>2852.204</t>
+        </is>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>Contractor Employee Security Screening</t>
+        </is>
+      </c>
+      <c r="E49" s="10" t="inlineStr">
+        <is>
+          <t>DoJ contractor employees must undergo security screening.</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" s="10" t="inlineStr">
+        <is>
+          <t>MOCK-Suppressors_5.56_NATO</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>JAR</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>JAR 2852.209-71</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>2852.209</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Standards of Conduct</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>DoJ standards of conduct — apply to your on-site employees.</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-Suppressors_5.56_NATO</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>NFS</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>NFS 1852.204-76</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>1852.204</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>Security Requirements for Unclassified Information Technology Resources</t>
+        </is>
+      </c>
+      <c r="E51" s="10" t="inlineStr">
+        <is>
+          <t>NASA IT-security requirements for unclassified systems.</t>
+        </is>
+      </c>
+      <c r="F51" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="10" t="inlineStr">
+        <is>
+          <t>MOCK-DetaClad_Explosion_Clad_Metal_made_up_of</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>NFS</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>NFS 1852.223-70</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>1852.223</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Safety and Health</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Maintain a written Safety and Health plan.</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-DetaClad_Explosion_Clad_Metal_made_up_of</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>NFS</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>NFS 1852.225-70</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>1852.225</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Export Licenses</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Handle export licensing for items subject to ITAR/EAR.</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-DetaClad_Explosion_Clad_Metal_made_up_of</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>NFS</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>NFS 1852.227-11</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>1852.227</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Patent Rights — Ownership by the Contractor</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Contractor may retain title to inventions (Bayh-Dole implementation).</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-DetaClad_Explosion_Clad_Metal_made_up_of</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>NFS</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>NFS 1852.245-70</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>1852.245</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Contractor Requests for Government-Owned Equipment</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Rules for requesting and using NASA-owned equipment.</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-DetaClad_Explosion_Clad_Metal_made_up_of</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>NFS</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>NFS 1852.246-70</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>1852.246</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Mission Critical Space System Personnel Reliability Program</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Mission-critical space system personnel reliability program.</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-DetaClad_Explosion_Clad_Metal_made_up_of</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="9" t="inlineStr">
+        <is>
+          <t>NMCARS</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>NMCARS 5252.204-9400</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>5252.204</t>
+        </is>
+      </c>
+      <c r="D57" s="10" t="inlineStr">
+        <is>
+          <t>Contractor Access to Federally-Controlled Facilities</t>
+        </is>
+      </c>
+      <c r="E57" s="10" t="inlineStr">
+        <is>
+          <t>Navy contractor access to federally-controlled facilities.</t>
+        </is>
+      </c>
+      <c r="F57" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="G57" s="10" t="inlineStr">
+        <is>
+          <t>MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>NMCARS</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>NMCARS 5252.222-9300</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>5252.222</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Contractor Personnel Access to Work Sites</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Navy contractor personnel access to Navy work sites.</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>NMCARS</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>NMCARS 5252.223-9400</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>5252.223</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>Accident Reporting and Investigation</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>Report accidents/incidents to the Navy per this clause.</t>
+        </is>
+      </c>
+      <c r="F59" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>NMCARS</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>NMCARS 5252.242-9115</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>5252.242</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Technical Instructions</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Comply with technical instructions issued during performance.</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="9" t="inlineStr">
+        <is>
+          <t>USC</t>
+        </is>
+      </c>
+      <c r="B61" s="9" t="inlineStr">
+        <is>
+          <t>USC 10.4862</t>
+        </is>
+      </c>
+      <c r="C61" s="9" t="inlineStr">
+        <is>
+          <t>10.4862</t>
+        </is>
+      </c>
+      <c r="D61" s="10" t="inlineStr"/>
+      <c r="E61" s="10" t="inlineStr"/>
+      <c r="F61" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="G61" s="10" t="inlineStr">
+        <is>
+          <t>MOCK-BALLAST_LEAD, MOCK-CO2_Laser_Cutter___Engraver, MOCK-Metalwork_for_the_CLB_TCB_Unit_11_System, MOCK-PRESSURE_INTENSIFIER_UNIT, MOCK-Synopsis___Solicitation_for_CHUTE_ASSY__, MOCK-USNS_NEWPORT_HYDRAULIC_HOSE_REPLACEMENT, MOCK-USNS_NEWPORT_STERN_RAMP_MATERIAL, MOCK-Wheel__Solid_Rubber, SPE7L026T0325, SPE7L126T679S, SPE7L126T681K, SPE7L126T681X, SPE7L326Q1121, SPE7L326T035G, SPE7L326T036J, SPE7L326T061D, SPE7L326T062R, SPE7L326T062U, SPE7L326U0564, SPE7L426T4775, SPE7L426T4794, SPE7L426T5025, SPE7L426T5032, SPE7L426T5040, SPE7L426T5042, SPE7L526T3717, SPE7L726T3634, SPE8E426T1739, SPE8E426T1740, SPE8E426T1741, SPE8E426T1742, SPE8E426T1743, SPE8E526T2951, SPE8E526T3173, SPE8E926T2719</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AO61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -9125,7 +11264,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9193,7 +11332,7 @@
       <c r="D2" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="E2" s="9" t="n">
+      <c r="E2" s="12" t="n">
         <v>0.9743589743589743</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
@@ -9221,7 +11360,7 @@
       <c r="D3" s="8" t="n">
         <v>28</v>
       </c>
-      <c r="E3" s="10" t="n">
+      <c r="E3" s="13" t="n">
         <v>0.717948717948718</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -9249,7 +11388,7 @@
       <c r="D4" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="E4" s="9" t="n">
+      <c r="E4" s="12" t="n">
         <v>0.6410256410256411</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
@@ -9277,7 +11416,7 @@
       <c r="D5" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="13" t="n">
         <v>0.5384615384615384</v>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -9305,7 +11444,7 @@
       <c r="D6" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="E6" s="9" t="n">
+      <c r="E6" s="12" t="n">
         <v>0.5384615384615384</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -9333,7 +11472,7 @@
       <c r="D7" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="13" t="n">
         <v>0.3333333333333333</v>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -9361,7 +11500,7 @@
       <c r="D8" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="E8" s="9" t="n">
+      <c r="E8" s="12" t="n">
         <v>0.3333333333333333</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -9389,7 +11528,7 @@
       <c r="D9" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="13" t="n">
         <v>0.3333333333333333</v>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -9417,7 +11556,7 @@
       <c r="D10" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="E10" s="9" t="n">
+      <c r="E10" s="12" t="n">
         <v>0.2307692307692308</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -9445,7 +11584,7 @@
       <c r="D11" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="13" t="n">
         <v>0.2051282051282051</v>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -9473,7 +11612,7 @@
       <c r="D12" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="E12" s="9" t="n">
+      <c r="E12" s="12" t="n">
         <v>0.2051282051282051</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -9501,7 +11640,7 @@
       <c r="D13" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="13" t="n">
         <v>0.1538461538461539</v>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -9529,7 +11668,7 @@
       <c r="D14" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="E14" s="9" t="n">
+      <c r="E14" s="12" t="n">
         <v>0.1538461538461539</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -9557,7 +11696,7 @@
       <c r="D15" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E15" s="13" t="n">
         <v>0.1538461538461539</v>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -9585,7 +11724,7 @@
       <c r="D16" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="E16" s="9" t="n">
+      <c r="E16" s="12" t="n">
         <v>0.1538461538461539</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -9613,7 +11752,7 @@
       <c r="D17" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E17" s="13" t="n">
         <v>0.1538461538461539</v>
       </c>
       <c r="F17" s="7" t="inlineStr">
@@ -9641,7 +11780,7 @@
       <c r="D18" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="E18" s="9" t="n">
+      <c r="E18" s="12" t="n">
         <v>0.1025641025641026</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -9669,7 +11808,7 @@
       <c r="D19" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="E19" s="10" t="n">
+      <c r="E19" s="13" t="n">
         <v>0.1025641025641026</v>
       </c>
       <c r="F19" s="7" t="inlineStr">
@@ -9697,7 +11836,7 @@
       <c r="D20" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E20" s="9" t="n">
+      <c r="E20" s="12" t="n">
         <v>0.05128205128205128</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -9725,7 +11864,7 @@
       <c r="D21" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E21" s="10" t="n">
+      <c r="E21" s="13" t="n">
         <v>0.05128205128205128</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
@@ -9753,7 +11892,7 @@
       <c r="D22" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E22" s="9" t="n">
+      <c r="E22" s="12" t="n">
         <v>0.05128205128205128</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -9781,7 +11920,7 @@
       <c r="D23" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E23" s="10" t="n">
+      <c r="E23" s="13" t="n">
         <v>0.05128205128205128</v>
       </c>
       <c r="F23" s="7" t="inlineStr">
@@ -9809,7 +11948,7 @@
       <c r="D24" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="9" t="n">
+      <c r="E24" s="12" t="n">
         <v>0.02564102564102564</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -9823,7 +11962,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12152,7 +14291,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00888888"/>

</xml_diff>